<commit_message>
split tables by Period
</commit_message>
<xml_diff>
--- a/data/source/GSSPs.xlsx
+++ b/data/source/GSSPs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/work/ics/gssps/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED93A50A-8E8B-1247-B497-66E22D3EF178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C43F8D-ABE3-6D47-81EB-528960C07475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="720" windowWidth="43300" windowHeight="27100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1800" yWindow="720" windowWidth="43300" windowHeight="27100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GSSPs" sheetId="1" r:id="rId1"/>
@@ -4416,11 +4416,6 @@
     <t>https://doi.org/10.18814/epiiugs/2009/v32i4/001</t>
   </si>
   <si>
-    <t>https://doi.org/10.18814/epiiugs/2008/v31i2/016
-https://doi.org/10.18814/epiiugs/2018/018016
-https://stratigraphy.org/gssps/files/meghalayan.pdf</t>
-  </si>
-  <si>
     <t>https://doi.org/10.18814/epiiugs/1985/v8i2/009
 https://doi.org/10.18814/epiiugs/2012/v35i3/001
 https://doi.org/10.1016/j.quaint.2019.05.018</t>
@@ -4681,6 +4676,10 @@
   </si>
   <si>
     <t>https://doi.org/10.18814/epiiugs/2020/020080</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.18814/epiiugs/2008/v31i2/016
+https://doi.org/10.18814/epiiugs/2018/018016</t>
   </si>
 </sst>
 </file>
@@ -5094,7 +5093,7 @@
         <v>14</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -5126,7 +5125,7 @@
         <v>14</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -5158,7 +5157,7 @@
         <v>24</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>726</v>
+        <v>793</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -5223,7 +5222,7 @@
         <v>37</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -5290,7 +5289,7 @@
         <v>49</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="102" customHeight="1" x14ac:dyDescent="0.2">
@@ -5325,7 +5324,7 @@
         <v>56</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -5360,7 +5359,7 @@
         <v>63</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -5395,7 +5394,7 @@
         <v>70</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -5430,7 +5429,7 @@
         <v>70</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -5465,7 +5464,7 @@
         <v>81</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -5500,7 +5499,7 @@
         <v>87</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -5590,7 +5589,7 @@
         <v>101</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -5660,7 +5659,7 @@
         <v>114</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="102" customHeight="1" x14ac:dyDescent="0.2">
@@ -5753,7 +5752,7 @@
         <v>129</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -5788,7 +5787,7 @@
         <v>81</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -5823,7 +5822,7 @@
         <v>142</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -5858,7 +5857,7 @@
         <v>142</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -5893,7 +5892,7 @@
         <v>153</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -5928,7 +5927,7 @@
         <v>159</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -5998,7 +5997,7 @@
         <v>173</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -6068,7 +6067,7 @@
         <v>81</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -6103,7 +6102,7 @@
         <v>191</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -6433,7 +6432,7 @@
         <v>101</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -6468,7 +6467,7 @@
         <v>70</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -6503,7 +6502,7 @@
         <v>243</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -6538,7 +6537,7 @@
         <v>249</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -6573,7 +6572,7 @@
         <v>70</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -6608,7 +6607,7 @@
         <v>260</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -6689,7 +6688,7 @@
         <v>142</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="136" customHeight="1" x14ac:dyDescent="0.2">
@@ -6724,7 +6723,7 @@
         <v>249</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -6756,7 +6755,7 @@
         <v>279</v>
       </c>
       <c r="K54" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -6788,7 +6787,7 @@
         <v>279</v>
       </c>
       <c r="K55" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -6823,7 +6822,7 @@
         <v>159</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -6858,7 +6857,7 @@
         <v>249</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -6893,7 +6892,7 @@
         <v>302</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -6928,7 +6927,7 @@
         <v>159</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -6963,7 +6962,7 @@
         <v>159</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -6998,7 +6997,7 @@
         <v>159</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -7125,7 +7124,7 @@
         <v>101</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -7226,7 +7225,7 @@
         <v>101</v>
       </c>
       <c r="K69" s="6" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7281,7 +7280,7 @@
         <v>142</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -7313,7 +7312,7 @@
         <v>367</v>
       </c>
       <c r="K72" s="6" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -7345,7 +7344,7 @@
         <v>373</v>
       </c>
       <c r="K73" s="6" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="74" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7377,7 +7376,7 @@
         <v>379</v>
       </c>
       <c r="K74" s="6" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -7409,7 +7408,7 @@
         <v>385</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7441,7 +7440,7 @@
         <v>391</v>
       </c>
       <c r="K76" s="6" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7473,7 +7472,7 @@
         <v>397</v>
       </c>
       <c r="K77" s="6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -7505,7 +7504,7 @@
         <v>403</v>
       </c>
       <c r="K78" s="6" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="153" customHeight="1" x14ac:dyDescent="0.2">
@@ -7537,7 +7536,7 @@
         <v>408</v>
       </c>
       <c r="K79" s="6" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -7569,7 +7568,7 @@
         <v>413</v>
       </c>
       <c r="K80" s="6" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="53" customHeight="1" x14ac:dyDescent="0.2">
@@ -7601,7 +7600,7 @@
         <v>418</v>
       </c>
       <c r="K81" s="6" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="53" customHeight="1" x14ac:dyDescent="0.2">
@@ -7633,7 +7632,7 @@
         <v>418</v>
       </c>
       <c r="K82" s="6" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="53" customHeight="1" x14ac:dyDescent="0.2">
@@ -7665,7 +7664,7 @@
         <v>418</v>
       </c>
       <c r="K83" s="6" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="204" customHeight="1" x14ac:dyDescent="0.2">
@@ -7682,7 +7681,7 @@
         <v>605</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>426</v>
@@ -7700,7 +7699,7 @@
         <v>418</v>
       </c>
       <c r="K84" s="6" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="102" customHeight="1" x14ac:dyDescent="0.2">
@@ -7732,7 +7731,7 @@
         <v>433</v>
       </c>
       <c r="K85" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="102" customHeight="1" x14ac:dyDescent="0.2">
@@ -7764,7 +7763,7 @@
         <v>438</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="38" customHeight="1" x14ac:dyDescent="0.2">
@@ -7796,7 +7795,7 @@
         <v>413</v>
       </c>
       <c r="K87" s="6" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7828,7 +7827,7 @@
         <v>447</v>
       </c>
       <c r="K88" s="6" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7860,7 +7859,7 @@
         <v>447</v>
       </c>
       <c r="K89" s="6" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7892,7 +7891,7 @@
         <v>191</v>
       </c>
       <c r="K90" s="6" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7924,7 +7923,7 @@
         <v>460</v>
       </c>
       <c r="K91" s="6" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -7956,7 +7955,7 @@
         <v>87</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -7988,7 +7987,7 @@
         <v>191</v>
       </c>
       <c r="K93" s="6" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -8020,7 +8019,7 @@
         <v>70</v>
       </c>
       <c r="K94" s="6" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -8075,7 +8074,7 @@
         <v>129</v>
       </c>
       <c r="K96" s="6" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -8139,7 +8138,7 @@
         <v>142</v>
       </c>
       <c r="K98" s="6" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -8171,7 +8170,7 @@
         <v>447</v>
       </c>
       <c r="K99" s="6" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -8286,7 +8285,7 @@
         <v>114</v>
       </c>
       <c r="K104" s="6" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -8340,7 +8339,7 @@
       <c r="G106" s="7"/>
       <c r="J106" s="7"/>
       <c r="K106" s="6" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8364,7 +8363,7 @@
         <v>367</v>
       </c>
       <c r="K107" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8388,7 +8387,7 @@
         <v>367</v>
       </c>
       <c r="K108" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8412,7 +8411,7 @@
         <v>367</v>
       </c>
       <c r="K109" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8436,7 +8435,7 @@
         <v>367</v>
       </c>
       <c r="K110" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8460,7 +8459,7 @@
         <v>367</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8484,7 +8483,7 @@
         <v>367</v>
       </c>
       <c r="K112" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8508,7 +8507,7 @@
         <v>367</v>
       </c>
       <c r="K113" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8532,7 +8531,7 @@
         <v>367</v>
       </c>
       <c r="K114" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8556,7 +8555,7 @@
         <v>524</v>
       </c>
       <c r="K115" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8580,7 +8579,7 @@
         <v>524</v>
       </c>
       <c r="K116" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="23" customHeight="1" x14ac:dyDescent="0.2">
@@ -8604,7 +8603,7 @@
         <v>524</v>
       </c>
       <c r="K117" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -8636,7 +8635,7 @@
         <v>41</v>
       </c>
       <c r="K118" s="2" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="119" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>